<commit_message>
feat: configurable WhatsApp notification templates with live preview
- Add wa_checkin_normal, wa_checkin_late, wa_checkout to settings
- notificationService loads templates from DB with placeholder replacement
- WhatsAppSection: template editor with textarea, preview, save & reset
- GET /api/settings/templates/defaults endpoint for default values
- Placeholders: {nama}, {waktu}, {tanggal}, {status}, {kelas}
</commit_message>
<xml_diff>
--- a/backend/uploads/templates/template-import-siswa.xlsx
+++ b/backend/uploads/templates/template-import-siswa.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Siswa" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,11 +397,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:G2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -414,43 +418,45 @@
       <c r="C1" t="str">
         <v>Kelas</v>
       </c>
+      <c r="D1" t="str">
+        <v>Nama Orang Tua</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Password</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Nomer HP</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2024001</v>
+        <v>260001</v>
       </c>
       <c r="B2" t="str">
-        <v>Andi Pratama</v>
+        <v>Budi Santoso</v>
       </c>
       <c r="C2" t="str">
-        <v>X-A</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2024002</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Budi Santoso</v>
-      </c>
-      <c r="C3" t="str">
-        <v>X-A</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>2024003</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Citra Dewi</v>
-      </c>
-      <c r="C4" t="str">
-        <v>X-B</v>
+        <v>X IPA 1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Siti Aminah</v>
+      </c>
+      <c r="E2" t="str">
+        <v>siti.ortu@example.com</v>
+      </c>
+      <c r="F2" t="str">
+        <v>260001HadirQ</v>
+      </c>
+      <c r="G2" t="str">
+        <v>08123456789</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>